<commit_message>
Polish test cases and bug reports
</commit_message>
<xml_diff>
--- a/Bug_Reports/bug_reports.xlsx
+++ b/Bug_Reports/bug_reports.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\projekt-manual-testing-saucedemo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\manual-testing-ecommerce-app\Bug_Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{575B7283-7DE4-49A9-98E7-746E23C4F596}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6CA2FD1-65BC-4515-AF85-E89DFD9236AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9510" yWindow="0" windowWidth="9780" windowHeight="11370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -75,13 +75,7 @@
 4. Open the Cart page.</t>
   </si>
   <si>
-    <t>Expected result</t>
-  </si>
-  <si>
     <t>The selected products are added to the shopping cart. The "Add to cart" button changes to "Remove" for each selected product. The shopping cart badge displays the correct number of added products.</t>
-  </si>
-  <si>
-    <t>The "Add to cart" button does not change to "Remove" for the affected products. The selected products are not addded to the shopping cart.</t>
   </si>
   <si>
     <t>High</t>
@@ -141,9 +135,6 @@
     <t>The product details page displays the correct product name, description, image and price.</t>
   </si>
   <si>
-    <t>The product details displays "ITEM NOT FOUND", an incrorrect description, an incorrect image and an invalid price ($√-1).</t>
-  </si>
-  <si>
     <t>BUG-005</t>
   </si>
   <si>
@@ -162,19 +153,36 @@
     <t>The user can enter values into the First Name, Last Name and Zip/Postal Code fields and proceed to Checkout: Overview.</t>
   </si>
   <si>
-    <t>The user cannot enterany value into the Last Name field. As a result, the user cannot continue to Chechkout: Overview.</t>
+    <t>The "Add to cart" button does not change to "Remove" for the affected products. The selected products are not added to the shopping cart.</t>
+  </si>
+  <si>
+    <t>The product details displays "ITEM NOT FOUND", an incorrect description, an incorrect image and an invalid price ($√-1).</t>
+  </si>
+  <si>
+    <t>The user cannot enter any value into the Last Name field. As a result, the user cannot continue to Checkout: Overview.</t>
+  </si>
+  <si>
+    <t>Expected Result</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -212,13 +220,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -287,7 +298,7 @@
     <tableColumn id="3" xr3:uid="{FE39D608-B53D-4C75-9A1E-18AB4027675F}" name="Environment" dataDxfId="7"/>
     <tableColumn id="4" xr3:uid="{57154840-9694-4882-91DE-8A4ED85F5139}" name="Preconditions" dataDxfId="6"/>
     <tableColumn id="5" xr3:uid="{80BF309A-0E61-47FF-B881-DCA8248BCA3A}" name="Steps to Reproduce" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{10C8065C-2898-4A57-A922-518A0714738D}" name="Expected result" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{10C8065C-2898-4A57-A922-518A0714738D}" name="Expected Result" dataDxfId="4"/>
     <tableColumn id="7" xr3:uid="{6175F95B-D5C5-4D5E-997F-50A39D49DAB7}" name="Actual Result" dataDxfId="3"/>
     <tableColumn id="8" xr3:uid="{272C3AC8-D799-423B-931E-DCB8EACCB4E4}" name="Severity" dataDxfId="2"/>
     <tableColumn id="9" xr3:uid="{BB1D0787-C783-4824-AA0B-65F813E84111}" name="Priority" dataDxfId="1"/>
@@ -591,8 +602,8 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>14</v>
+      <c r="F1" s="3" t="s">
+        <v>40</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>5</v>
@@ -624,27 +635,27 @@
         <v>13</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="G2" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="I2" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="130.5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>10</v>
@@ -653,30 +664,30 @@
         <v>12</v>
       </c>
       <c r="E3" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="H3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="J3" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="87" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>10</v>
@@ -685,30 +696,30 @@
         <v>12</v>
       </c>
       <c r="E4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="F4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="H4" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="87" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>30</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>32</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>10</v>
@@ -717,58 +728,58 @@
         <v>12</v>
       </c>
       <c r="E5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>33</v>
-      </c>
       <c r="G5" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="87" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="H6" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>